<commit_message>
YHAAO-12232 APM IB -- 支持LCS贴码YHAAO-12286 贴码准备
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/uaa/userAccount/UserAccountImport_Template.xlsx
+++ b/src/src/main/webapp/portal/uaa/userAccount/UserAccountImport_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212670825\Desktop\APM\Git\hc-apm-web\src\src\main\webapp\portal\uaa\userAccount\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\zp\code\web\hc-apm-web-ib\src\src\main\webapp\portal\uaa\userAccount\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCA2815-638A-4FB5-A2DC-30710618B7B9}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA916DC9-9AB8-47D8-B24D-0BE529742578}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datalist" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>所属集团</t>
   </si>
@@ -294,12 +294,18 @@
   <si>
     <t>标签</t>
   </si>
+  <si>
+    <t>所属代理商</t>
+  </si>
+  <si>
+    <t>XXXX</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -317,6 +323,12 @@
       <color indexed="8"/>
       <name val="宋体"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="GE Inspira Sans"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -339,7 +351,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -452,11 +464,52 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="11"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="11"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -468,11 +521,9 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -488,6 +539,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1626,8 +1686,8 @@
     <col min="11" max="12" width="8.77734375" style="1" customWidth="1"/>
     <col min="13" max="13" width="24.6640625" style="1" customWidth="1"/>
     <col min="14" max="17" width="30" style="1" customWidth="1"/>
-    <col min="18" max="18" width="32.6640625" style="1" customWidth="1"/>
-    <col min="19" max="258" width="8.77734375" style="1" customWidth="1"/>
+    <col min="18" max="19" width="32.6640625" style="1" customWidth="1"/>
+    <col min="20" max="258" width="8.77734375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:258" ht="30.75" customHeight="1">
@@ -1685,246 +1745,248 @@
       <c r="R1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="7"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
-      <c r="AA1" s="10"/>
-      <c r="AB1" s="10"/>
-      <c r="AC1" s="10"/>
-      <c r="AD1" s="10"/>
-      <c r="AE1" s="10"/>
-      <c r="AF1" s="10"/>
-      <c r="AG1" s="10"/>
-      <c r="AH1" s="10"/>
-      <c r="AI1" s="10"/>
-      <c r="AJ1" s="10"/>
-      <c r="AK1" s="10"/>
-      <c r="AL1" s="10"/>
-      <c r="AM1" s="10"/>
-      <c r="AN1" s="10"/>
-      <c r="AO1" s="10"/>
-      <c r="AP1" s="10"/>
-      <c r="AQ1" s="10"/>
-      <c r="AR1" s="10"/>
-      <c r="AS1" s="10"/>
-      <c r="AT1" s="10"/>
-      <c r="AU1" s="10"/>
-      <c r="AV1" s="10"/>
-      <c r="AW1" s="10"/>
-      <c r="AX1" s="10"/>
-      <c r="AY1" s="10"/>
-      <c r="AZ1" s="10"/>
-      <c r="BA1" s="10"/>
-      <c r="BB1" s="10"/>
-      <c r="BC1" s="10"/>
-      <c r="BD1" s="10"/>
-      <c r="BE1" s="10"/>
-      <c r="BF1" s="10"/>
-      <c r="BG1" s="10"/>
-      <c r="BH1" s="10"/>
-      <c r="BI1" s="10"/>
-      <c r="BJ1" s="10"/>
-      <c r="BK1" s="10"/>
-      <c r="BL1" s="10"/>
-      <c r="BM1" s="10"/>
-      <c r="BN1" s="10"/>
-      <c r="BO1" s="10"/>
-      <c r="BP1" s="10"/>
-      <c r="BQ1" s="10"/>
-      <c r="BR1" s="10"/>
-      <c r="BS1" s="10"/>
-      <c r="BT1" s="10"/>
-      <c r="BU1" s="10"/>
-      <c r="BV1" s="10"/>
-      <c r="BW1" s="10"/>
-      <c r="BX1" s="10"/>
-      <c r="BY1" s="10"/>
-      <c r="BZ1" s="10"/>
-      <c r="CA1" s="10"/>
-      <c r="CB1" s="10"/>
-      <c r="CC1" s="10"/>
-      <c r="CD1" s="10"/>
-      <c r="CE1" s="10"/>
-      <c r="CF1" s="10"/>
-      <c r="CG1" s="10"/>
-      <c r="CH1" s="10"/>
-      <c r="CI1" s="10"/>
-      <c r="CJ1" s="10"/>
-      <c r="CK1" s="10"/>
-      <c r="CL1" s="10"/>
-      <c r="CM1" s="10"/>
-      <c r="CN1" s="10"/>
-      <c r="CO1" s="10"/>
-      <c r="CP1" s="10"/>
-      <c r="CQ1" s="10"/>
-      <c r="CR1" s="10"/>
-      <c r="CS1" s="10"/>
-      <c r="CT1" s="10"/>
-      <c r="CU1" s="10"/>
-      <c r="CV1" s="10"/>
-      <c r="CW1" s="10"/>
-      <c r="CX1" s="10"/>
-      <c r="CY1" s="10"/>
-      <c r="CZ1" s="10"/>
-      <c r="DA1" s="10"/>
-      <c r="DB1" s="10"/>
-      <c r="DC1" s="10"/>
-      <c r="DD1" s="10"/>
-      <c r="DE1" s="10"/>
-      <c r="DF1" s="10"/>
-      <c r="DG1" s="10"/>
-      <c r="DH1" s="10"/>
-      <c r="DI1" s="10"/>
-      <c r="DJ1" s="10"/>
-      <c r="DK1" s="10"/>
-      <c r="DL1" s="10"/>
-      <c r="DM1" s="10"/>
-      <c r="DN1" s="10"/>
-      <c r="DO1" s="10"/>
-      <c r="DP1" s="10"/>
-      <c r="DQ1" s="10"/>
-      <c r="DR1" s="10"/>
-      <c r="DS1" s="10"/>
-      <c r="DT1" s="10"/>
-      <c r="DU1" s="10"/>
-      <c r="DV1" s="10"/>
-      <c r="DW1" s="10"/>
-      <c r="DX1" s="10"/>
-      <c r="DY1" s="10"/>
-      <c r="DZ1" s="10"/>
-      <c r="EA1" s="10"/>
-      <c r="EB1" s="10"/>
-      <c r="EC1" s="10"/>
-      <c r="ED1" s="10"/>
-      <c r="EE1" s="10"/>
-      <c r="EF1" s="10"/>
-      <c r="EG1" s="10"/>
-      <c r="EH1" s="10"/>
-      <c r="EI1" s="10"/>
-      <c r="EJ1" s="10"/>
-      <c r="EK1" s="10"/>
-      <c r="EL1" s="10"/>
-      <c r="EM1" s="10"/>
-      <c r="EN1" s="10"/>
-      <c r="EO1" s="10"/>
-      <c r="EP1" s="10"/>
-      <c r="EQ1" s="10"/>
-      <c r="ER1" s="10"/>
-      <c r="ES1" s="10"/>
-      <c r="ET1" s="10"/>
-      <c r="EU1" s="10"/>
-      <c r="EV1" s="10"/>
-      <c r="EW1" s="10"/>
-      <c r="EX1" s="10"/>
-      <c r="EY1" s="10"/>
-      <c r="EZ1" s="10"/>
-      <c r="FA1" s="10"/>
-      <c r="FB1" s="10"/>
-      <c r="FC1" s="10"/>
-      <c r="FD1" s="10"/>
-      <c r="FE1" s="10"/>
-      <c r="FF1" s="10"/>
-      <c r="FG1" s="10"/>
-      <c r="FH1" s="10"/>
-      <c r="FI1" s="10"/>
-      <c r="FJ1" s="10"/>
-      <c r="FK1" s="10"/>
-      <c r="FL1" s="10"/>
-      <c r="FM1" s="10"/>
-      <c r="FN1" s="10"/>
-      <c r="FO1" s="10"/>
-      <c r="FP1" s="10"/>
-      <c r="FQ1" s="10"/>
-      <c r="FR1" s="10"/>
-      <c r="FS1" s="10"/>
-      <c r="FT1" s="10"/>
-      <c r="FU1" s="10"/>
-      <c r="FV1" s="10"/>
-      <c r="FW1" s="10"/>
-      <c r="FX1" s="10"/>
-      <c r="FY1" s="10"/>
-      <c r="FZ1" s="10"/>
-      <c r="GA1" s="10"/>
-      <c r="GB1" s="10"/>
-      <c r="GC1" s="10"/>
-      <c r="GD1" s="10"/>
-      <c r="GE1" s="10"/>
-      <c r="GF1" s="10"/>
-      <c r="GG1" s="10"/>
-      <c r="GH1" s="10"/>
-      <c r="GI1" s="10"/>
-      <c r="GJ1" s="10"/>
-      <c r="GK1" s="10"/>
-      <c r="GL1" s="10"/>
-      <c r="GM1" s="10"/>
-      <c r="GN1" s="10"/>
-      <c r="GO1" s="10"/>
-      <c r="GP1" s="10"/>
-      <c r="GQ1" s="10"/>
-      <c r="GR1" s="10"/>
-      <c r="GS1" s="10"/>
-      <c r="GT1" s="10"/>
-      <c r="GU1" s="10"/>
-      <c r="GV1" s="10"/>
-      <c r="GW1" s="10"/>
-      <c r="GX1" s="10"/>
-      <c r="GY1" s="10"/>
-      <c r="GZ1" s="10"/>
-      <c r="HA1" s="10"/>
-      <c r="HB1" s="10"/>
-      <c r="HC1" s="10"/>
-      <c r="HD1" s="10"/>
-      <c r="HE1" s="10"/>
-      <c r="HF1" s="10"/>
-      <c r="HG1" s="10"/>
-      <c r="HH1" s="10"/>
-      <c r="HI1" s="10"/>
-      <c r="HJ1" s="10"/>
-      <c r="HK1" s="10"/>
-      <c r="HL1" s="10"/>
-      <c r="HM1" s="10"/>
-      <c r="HN1" s="10"/>
-      <c r="HO1" s="10"/>
-      <c r="HP1" s="10"/>
-      <c r="HQ1" s="10"/>
-      <c r="HR1" s="10"/>
-      <c r="HS1" s="10"/>
-      <c r="HT1" s="10"/>
-      <c r="HU1" s="10"/>
-      <c r="HV1" s="10"/>
-      <c r="HW1" s="10"/>
-      <c r="HX1" s="10"/>
-      <c r="HY1" s="10"/>
-      <c r="HZ1" s="10"/>
-      <c r="IA1" s="10"/>
-      <c r="IB1" s="10"/>
-      <c r="IC1" s="10"/>
-      <c r="ID1" s="10"/>
-      <c r="IE1" s="10"/>
-      <c r="IF1" s="10"/>
-      <c r="IG1" s="10"/>
-      <c r="IH1" s="10"/>
-      <c r="II1" s="10"/>
-      <c r="IJ1" s="10"/>
-      <c r="IK1" s="10"/>
-      <c r="IL1" s="10"/>
-      <c r="IM1" s="10"/>
-      <c r="IN1" s="10"/>
-      <c r="IO1" s="10"/>
-      <c r="IP1" s="10"/>
-      <c r="IQ1" s="10"/>
-      <c r="IR1" s="10"/>
-      <c r="IS1" s="10"/>
-      <c r="IT1" s="10"/>
-      <c r="IU1" s="10"/>
-      <c r="IV1" s="10"/>
-      <c r="IW1" s="10"/>
-      <c r="IX1" s="12"/>
+      <c r="S1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
+      <c r="AA1" s="8"/>
+      <c r="AB1" s="8"/>
+      <c r="AC1" s="8"/>
+      <c r="AD1" s="8"/>
+      <c r="AE1" s="8"/>
+      <c r="AF1" s="8"/>
+      <c r="AG1" s="8"/>
+      <c r="AH1" s="8"/>
+      <c r="AI1" s="8"/>
+      <c r="AJ1" s="8"/>
+      <c r="AK1" s="8"/>
+      <c r="AL1" s="8"/>
+      <c r="AM1" s="8"/>
+      <c r="AN1" s="8"/>
+      <c r="AO1" s="8"/>
+      <c r="AP1" s="8"/>
+      <c r="AQ1" s="8"/>
+      <c r="AR1" s="8"/>
+      <c r="AS1" s="8"/>
+      <c r="AT1" s="8"/>
+      <c r="AU1" s="8"/>
+      <c r="AV1" s="8"/>
+      <c r="AW1" s="8"/>
+      <c r="AX1" s="8"/>
+      <c r="AY1" s="8"/>
+      <c r="AZ1" s="8"/>
+      <c r="BA1" s="8"/>
+      <c r="BB1" s="8"/>
+      <c r="BC1" s="8"/>
+      <c r="BD1" s="8"/>
+      <c r="BE1" s="8"/>
+      <c r="BF1" s="8"/>
+      <c r="BG1" s="8"/>
+      <c r="BH1" s="8"/>
+      <c r="BI1" s="8"/>
+      <c r="BJ1" s="8"/>
+      <c r="BK1" s="8"/>
+      <c r="BL1" s="8"/>
+      <c r="BM1" s="8"/>
+      <c r="BN1" s="8"/>
+      <c r="BO1" s="8"/>
+      <c r="BP1" s="8"/>
+      <c r="BQ1" s="8"/>
+      <c r="BR1" s="8"/>
+      <c r="BS1" s="8"/>
+      <c r="BT1" s="8"/>
+      <c r="BU1" s="8"/>
+      <c r="BV1" s="8"/>
+      <c r="BW1" s="8"/>
+      <c r="BX1" s="8"/>
+      <c r="BY1" s="8"/>
+      <c r="BZ1" s="8"/>
+      <c r="CA1" s="8"/>
+      <c r="CB1" s="8"/>
+      <c r="CC1" s="8"/>
+      <c r="CD1" s="8"/>
+      <c r="CE1" s="8"/>
+      <c r="CF1" s="8"/>
+      <c r="CG1" s="8"/>
+      <c r="CH1" s="8"/>
+      <c r="CI1" s="8"/>
+      <c r="CJ1" s="8"/>
+      <c r="CK1" s="8"/>
+      <c r="CL1" s="8"/>
+      <c r="CM1" s="8"/>
+      <c r="CN1" s="8"/>
+      <c r="CO1" s="8"/>
+      <c r="CP1" s="8"/>
+      <c r="CQ1" s="8"/>
+      <c r="CR1" s="8"/>
+      <c r="CS1" s="8"/>
+      <c r="CT1" s="8"/>
+      <c r="CU1" s="8"/>
+      <c r="CV1" s="8"/>
+      <c r="CW1" s="8"/>
+      <c r="CX1" s="8"/>
+      <c r="CY1" s="8"/>
+      <c r="CZ1" s="8"/>
+      <c r="DA1" s="8"/>
+      <c r="DB1" s="8"/>
+      <c r="DC1" s="8"/>
+      <c r="DD1" s="8"/>
+      <c r="DE1" s="8"/>
+      <c r="DF1" s="8"/>
+      <c r="DG1" s="8"/>
+      <c r="DH1" s="8"/>
+      <c r="DI1" s="8"/>
+      <c r="DJ1" s="8"/>
+      <c r="DK1" s="8"/>
+      <c r="DL1" s="8"/>
+      <c r="DM1" s="8"/>
+      <c r="DN1" s="8"/>
+      <c r="DO1" s="8"/>
+      <c r="DP1" s="8"/>
+      <c r="DQ1" s="8"/>
+      <c r="DR1" s="8"/>
+      <c r="DS1" s="8"/>
+      <c r="DT1" s="8"/>
+      <c r="DU1" s="8"/>
+      <c r="DV1" s="8"/>
+      <c r="DW1" s="8"/>
+      <c r="DX1" s="8"/>
+      <c r="DY1" s="8"/>
+      <c r="DZ1" s="8"/>
+      <c r="EA1" s="8"/>
+      <c r="EB1" s="8"/>
+      <c r="EC1" s="8"/>
+      <c r="ED1" s="8"/>
+      <c r="EE1" s="8"/>
+      <c r="EF1" s="8"/>
+      <c r="EG1" s="8"/>
+      <c r="EH1" s="8"/>
+      <c r="EI1" s="8"/>
+      <c r="EJ1" s="8"/>
+      <c r="EK1" s="8"/>
+      <c r="EL1" s="8"/>
+      <c r="EM1" s="8"/>
+      <c r="EN1" s="8"/>
+      <c r="EO1" s="8"/>
+      <c r="EP1" s="8"/>
+      <c r="EQ1" s="8"/>
+      <c r="ER1" s="8"/>
+      <c r="ES1" s="8"/>
+      <c r="ET1" s="8"/>
+      <c r="EU1" s="8"/>
+      <c r="EV1" s="8"/>
+      <c r="EW1" s="8"/>
+      <c r="EX1" s="8"/>
+      <c r="EY1" s="8"/>
+      <c r="EZ1" s="8"/>
+      <c r="FA1" s="8"/>
+      <c r="FB1" s="8"/>
+      <c r="FC1" s="8"/>
+      <c r="FD1" s="8"/>
+      <c r="FE1" s="8"/>
+      <c r="FF1" s="8"/>
+      <c r="FG1" s="8"/>
+      <c r="FH1" s="8"/>
+      <c r="FI1" s="8"/>
+      <c r="FJ1" s="8"/>
+      <c r="FK1" s="8"/>
+      <c r="FL1" s="8"/>
+      <c r="FM1" s="8"/>
+      <c r="FN1" s="8"/>
+      <c r="FO1" s="8"/>
+      <c r="FP1" s="8"/>
+      <c r="FQ1" s="8"/>
+      <c r="FR1" s="8"/>
+      <c r="FS1" s="8"/>
+      <c r="FT1" s="8"/>
+      <c r="FU1" s="8"/>
+      <c r="FV1" s="8"/>
+      <c r="FW1" s="8"/>
+      <c r="FX1" s="8"/>
+      <c r="FY1" s="8"/>
+      <c r="FZ1" s="8"/>
+      <c r="GA1" s="8"/>
+      <c r="GB1" s="8"/>
+      <c r="GC1" s="8"/>
+      <c r="GD1" s="8"/>
+      <c r="GE1" s="8"/>
+      <c r="GF1" s="8"/>
+      <c r="GG1" s="8"/>
+      <c r="GH1" s="8"/>
+      <c r="GI1" s="8"/>
+      <c r="GJ1" s="8"/>
+      <c r="GK1" s="8"/>
+      <c r="GL1" s="8"/>
+      <c r="GM1" s="8"/>
+      <c r="GN1" s="8"/>
+      <c r="GO1" s="8"/>
+      <c r="GP1" s="8"/>
+      <c r="GQ1" s="8"/>
+      <c r="GR1" s="8"/>
+      <c r="GS1" s="8"/>
+      <c r="GT1" s="8"/>
+      <c r="GU1" s="8"/>
+      <c r="GV1" s="8"/>
+      <c r="GW1" s="8"/>
+      <c r="GX1" s="8"/>
+      <c r="GY1" s="8"/>
+      <c r="GZ1" s="8"/>
+      <c r="HA1" s="8"/>
+      <c r="HB1" s="8"/>
+      <c r="HC1" s="8"/>
+      <c r="HD1" s="8"/>
+      <c r="HE1" s="8"/>
+      <c r="HF1" s="8"/>
+      <c r="HG1" s="8"/>
+      <c r="HH1" s="8"/>
+      <c r="HI1" s="8"/>
+      <c r="HJ1" s="8"/>
+      <c r="HK1" s="8"/>
+      <c r="HL1" s="8"/>
+      <c r="HM1" s="8"/>
+      <c r="HN1" s="8"/>
+      <c r="HO1" s="8"/>
+      <c r="HP1" s="8"/>
+      <c r="HQ1" s="8"/>
+      <c r="HR1" s="8"/>
+      <c r="HS1" s="8"/>
+      <c r="HT1" s="8"/>
+      <c r="HU1" s="8"/>
+      <c r="HV1" s="8"/>
+      <c r="HW1" s="8"/>
+      <c r="HX1" s="8"/>
+      <c r="HY1" s="8"/>
+      <c r="HZ1" s="8"/>
+      <c r="IA1" s="8"/>
+      <c r="IB1" s="8"/>
+      <c r="IC1" s="8"/>
+      <c r="ID1" s="8"/>
+      <c r="IE1" s="8"/>
+      <c r="IF1" s="8"/>
+      <c r="IG1" s="8"/>
+      <c r="IH1" s="8"/>
+      <c r="II1" s="8"/>
+      <c r="IJ1" s="8"/>
+      <c r="IK1" s="8"/>
+      <c r="IL1" s="8"/>
+      <c r="IM1" s="8"/>
+      <c r="IN1" s="8"/>
+      <c r="IO1" s="8"/>
+      <c r="IP1" s="8"/>
+      <c r="IQ1" s="8"/>
+      <c r="IR1" s="8"/>
+      <c r="IS1" s="8"/>
+      <c r="IT1" s="8"/>
+      <c r="IU1" s="8"/>
+      <c r="IV1" s="8"/>
+      <c r="IW1" s="8"/>
+      <c r="IX1" s="10"/>
     </row>
     <row r="2" spans="1:258" ht="34.5" customHeight="1">
       <c r="A2" s="6" t="s">
@@ -1961,258 +2023,260 @@
       <c r="L2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="11"/>
-      <c r="U2" s="11"/>
-      <c r="V2" s="11"/>
-      <c r="W2" s="11"/>
-      <c r="X2" s="11"/>
-      <c r="Y2" s="11"/>
-      <c r="Z2" s="11"/>
-      <c r="AA2" s="11"/>
-      <c r="AB2" s="11"/>
-      <c r="AC2" s="11"/>
-      <c r="AD2" s="11"/>
-      <c r="AE2" s="11"/>
-      <c r="AF2" s="11"/>
-      <c r="AG2" s="11"/>
-      <c r="AH2" s="11"/>
-      <c r="AI2" s="11"/>
-      <c r="AJ2" s="11"/>
-      <c r="AK2" s="11"/>
-      <c r="AL2" s="11"/>
-      <c r="AM2" s="11"/>
-      <c r="AN2" s="11"/>
-      <c r="AO2" s="11"/>
-      <c r="AP2" s="11"/>
-      <c r="AQ2" s="11"/>
-      <c r="AR2" s="11"/>
-      <c r="AS2" s="11"/>
-      <c r="AT2" s="11"/>
-      <c r="AU2" s="11"/>
-      <c r="AV2" s="11"/>
-      <c r="AW2" s="11"/>
-      <c r="AX2" s="11"/>
-      <c r="AY2" s="11"/>
-      <c r="AZ2" s="11"/>
-      <c r="BA2" s="11"/>
-      <c r="BB2" s="11"/>
-      <c r="BC2" s="11"/>
-      <c r="BD2" s="11"/>
-      <c r="BE2" s="11"/>
-      <c r="BF2" s="11"/>
-      <c r="BG2" s="11"/>
-      <c r="BH2" s="11"/>
-      <c r="BI2" s="11"/>
-      <c r="BJ2" s="11"/>
-      <c r="BK2" s="11"/>
-      <c r="BL2" s="11"/>
-      <c r="BM2" s="11"/>
-      <c r="BN2" s="11"/>
-      <c r="BO2" s="11"/>
-      <c r="BP2" s="11"/>
-      <c r="BQ2" s="11"/>
-      <c r="BR2" s="11"/>
-      <c r="BS2" s="11"/>
-      <c r="BT2" s="11"/>
-      <c r="BU2" s="11"/>
-      <c r="BV2" s="11"/>
-      <c r="BW2" s="11"/>
-      <c r="BX2" s="11"/>
-      <c r="BY2" s="11"/>
-      <c r="BZ2" s="11"/>
-      <c r="CA2" s="11"/>
-      <c r="CB2" s="11"/>
-      <c r="CC2" s="11"/>
-      <c r="CD2" s="11"/>
-      <c r="CE2" s="11"/>
-      <c r="CF2" s="11"/>
-      <c r="CG2" s="11"/>
-      <c r="CH2" s="11"/>
-      <c r="CI2" s="11"/>
-      <c r="CJ2" s="11"/>
-      <c r="CK2" s="11"/>
-      <c r="CL2" s="11"/>
-      <c r="CM2" s="11"/>
-      <c r="CN2" s="11"/>
-      <c r="CO2" s="11"/>
-      <c r="CP2" s="11"/>
-      <c r="CQ2" s="11"/>
-      <c r="CR2" s="11"/>
-      <c r="CS2" s="11"/>
-      <c r="CT2" s="11"/>
-      <c r="CU2" s="11"/>
-      <c r="CV2" s="11"/>
-      <c r="CW2" s="11"/>
-      <c r="CX2" s="11"/>
-      <c r="CY2" s="11"/>
-      <c r="CZ2" s="11"/>
-      <c r="DA2" s="11"/>
-      <c r="DB2" s="11"/>
-      <c r="DC2" s="11"/>
-      <c r="DD2" s="11"/>
-      <c r="DE2" s="11"/>
-      <c r="DF2" s="11"/>
-      <c r="DG2" s="11"/>
-      <c r="DH2" s="11"/>
-      <c r="DI2" s="11"/>
-      <c r="DJ2" s="11"/>
-      <c r="DK2" s="11"/>
-      <c r="DL2" s="11"/>
-      <c r="DM2" s="11"/>
-      <c r="DN2" s="11"/>
-      <c r="DO2" s="11"/>
-      <c r="DP2" s="11"/>
-      <c r="DQ2" s="11"/>
-      <c r="DR2" s="11"/>
-      <c r="DS2" s="11"/>
-      <c r="DT2" s="11"/>
-      <c r="DU2" s="11"/>
-      <c r="DV2" s="11"/>
-      <c r="DW2" s="11"/>
-      <c r="DX2" s="11"/>
-      <c r="DY2" s="11"/>
-      <c r="DZ2" s="11"/>
-      <c r="EA2" s="11"/>
-      <c r="EB2" s="11"/>
-      <c r="EC2" s="11"/>
-      <c r="ED2" s="11"/>
-      <c r="EE2" s="11"/>
-      <c r="EF2" s="11"/>
-      <c r="EG2" s="11"/>
-      <c r="EH2" s="11"/>
-      <c r="EI2" s="11"/>
-      <c r="EJ2" s="11"/>
-      <c r="EK2" s="11"/>
-      <c r="EL2" s="11"/>
-      <c r="EM2" s="11"/>
-      <c r="EN2" s="11"/>
-      <c r="EO2" s="11"/>
-      <c r="EP2" s="11"/>
-      <c r="EQ2" s="11"/>
-      <c r="ER2" s="11"/>
-      <c r="ES2" s="11"/>
-      <c r="ET2" s="11"/>
-      <c r="EU2" s="11"/>
-      <c r="EV2" s="11"/>
-      <c r="EW2" s="11"/>
-      <c r="EX2" s="11"/>
-      <c r="EY2" s="11"/>
-      <c r="EZ2" s="11"/>
-      <c r="FA2" s="11"/>
-      <c r="FB2" s="11"/>
-      <c r="FC2" s="11"/>
-      <c r="FD2" s="11"/>
-      <c r="FE2" s="11"/>
-      <c r="FF2" s="11"/>
-      <c r="FG2" s="11"/>
-      <c r="FH2" s="11"/>
-      <c r="FI2" s="11"/>
-      <c r="FJ2" s="11"/>
-      <c r="FK2" s="11"/>
-      <c r="FL2" s="11"/>
-      <c r="FM2" s="11"/>
-      <c r="FN2" s="11"/>
-      <c r="FO2" s="11"/>
-      <c r="FP2" s="11"/>
-      <c r="FQ2" s="11"/>
-      <c r="FR2" s="11"/>
-      <c r="FS2" s="11"/>
-      <c r="FT2" s="11"/>
-      <c r="FU2" s="11"/>
-      <c r="FV2" s="11"/>
-      <c r="FW2" s="11"/>
-      <c r="FX2" s="11"/>
-      <c r="FY2" s="11"/>
-      <c r="FZ2" s="11"/>
-      <c r="GA2" s="11"/>
-      <c r="GB2" s="11"/>
-      <c r="GC2" s="11"/>
-      <c r="GD2" s="11"/>
-      <c r="GE2" s="11"/>
-      <c r="GF2" s="11"/>
-      <c r="GG2" s="11"/>
-      <c r="GH2" s="11"/>
-      <c r="GI2" s="11"/>
-      <c r="GJ2" s="11"/>
-      <c r="GK2" s="11"/>
-      <c r="GL2" s="11"/>
-      <c r="GM2" s="11"/>
-      <c r="GN2" s="11"/>
-      <c r="GO2" s="11"/>
-      <c r="GP2" s="11"/>
-      <c r="GQ2" s="11"/>
-      <c r="GR2" s="11"/>
-      <c r="GS2" s="11"/>
-      <c r="GT2" s="11"/>
-      <c r="GU2" s="11"/>
-      <c r="GV2" s="11"/>
-      <c r="GW2" s="11"/>
-      <c r="GX2" s="11"/>
-      <c r="GY2" s="11"/>
-      <c r="GZ2" s="11"/>
-      <c r="HA2" s="11"/>
-      <c r="HB2" s="11"/>
-      <c r="HC2" s="11"/>
-      <c r="HD2" s="11"/>
-      <c r="HE2" s="11"/>
-      <c r="HF2" s="11"/>
-      <c r="HG2" s="11"/>
-      <c r="HH2" s="11"/>
-      <c r="HI2" s="11"/>
-      <c r="HJ2" s="11"/>
-      <c r="HK2" s="11"/>
-      <c r="HL2" s="11"/>
-      <c r="HM2" s="11"/>
-      <c r="HN2" s="11"/>
-      <c r="HO2" s="11"/>
-      <c r="HP2" s="11"/>
-      <c r="HQ2" s="11"/>
-      <c r="HR2" s="11"/>
-      <c r="HS2" s="11"/>
-      <c r="HT2" s="11"/>
-      <c r="HU2" s="11"/>
-      <c r="HV2" s="11"/>
-      <c r="HW2" s="11"/>
-      <c r="HX2" s="11"/>
-      <c r="HY2" s="11"/>
-      <c r="HZ2" s="11"/>
-      <c r="IA2" s="11"/>
-      <c r="IB2" s="11"/>
-      <c r="IC2" s="11"/>
-      <c r="ID2" s="11"/>
-      <c r="IE2" s="11"/>
-      <c r="IF2" s="11"/>
-      <c r="IG2" s="11"/>
-      <c r="IH2" s="11"/>
-      <c r="II2" s="11"/>
-      <c r="IJ2" s="11"/>
-      <c r="IK2" s="11"/>
-      <c r="IL2" s="11"/>
-      <c r="IM2" s="11"/>
-      <c r="IN2" s="11"/>
-      <c r="IO2" s="11"/>
-      <c r="IP2" s="11"/>
-      <c r="IQ2" s="11"/>
-      <c r="IR2" s="11"/>
-      <c r="IS2" s="11"/>
-      <c r="IT2" s="11"/>
-      <c r="IU2" s="11"/>
-      <c r="IV2" s="11"/>
-      <c r="IW2" s="11"/>
-      <c r="IX2" s="13"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="9"/>
+      <c r="U2" s="9"/>
+      <c r="V2" s="9"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
+      <c r="AB2" s="9"/>
+      <c r="AC2" s="9"/>
+      <c r="AD2" s="9"/>
+      <c r="AE2" s="9"/>
+      <c r="AF2" s="9"/>
+      <c r="AG2" s="9"/>
+      <c r="AH2" s="9"/>
+      <c r="AI2" s="9"/>
+      <c r="AJ2" s="9"/>
+      <c r="AK2" s="9"/>
+      <c r="AL2" s="9"/>
+      <c r="AM2" s="9"/>
+      <c r="AN2" s="9"/>
+      <c r="AO2" s="9"/>
+      <c r="AP2" s="9"/>
+      <c r="AQ2" s="9"/>
+      <c r="AR2" s="9"/>
+      <c r="AS2" s="9"/>
+      <c r="AT2" s="9"/>
+      <c r="AU2" s="9"/>
+      <c r="AV2" s="9"/>
+      <c r="AW2" s="9"/>
+      <c r="AX2" s="9"/>
+      <c r="AY2" s="9"/>
+      <c r="AZ2" s="9"/>
+      <c r="BA2" s="9"/>
+      <c r="BB2" s="9"/>
+      <c r="BC2" s="9"/>
+      <c r="BD2" s="9"/>
+      <c r="BE2" s="9"/>
+      <c r="BF2" s="9"/>
+      <c r="BG2" s="9"/>
+      <c r="BH2" s="9"/>
+      <c r="BI2" s="9"/>
+      <c r="BJ2" s="9"/>
+      <c r="BK2" s="9"/>
+      <c r="BL2" s="9"/>
+      <c r="BM2" s="9"/>
+      <c r="BN2" s="9"/>
+      <c r="BO2" s="9"/>
+      <c r="BP2" s="9"/>
+      <c r="BQ2" s="9"/>
+      <c r="BR2" s="9"/>
+      <c r="BS2" s="9"/>
+      <c r="BT2" s="9"/>
+      <c r="BU2" s="9"/>
+      <c r="BV2" s="9"/>
+      <c r="BW2" s="9"/>
+      <c r="BX2" s="9"/>
+      <c r="BY2" s="9"/>
+      <c r="BZ2" s="9"/>
+      <c r="CA2" s="9"/>
+      <c r="CB2" s="9"/>
+      <c r="CC2" s="9"/>
+      <c r="CD2" s="9"/>
+      <c r="CE2" s="9"/>
+      <c r="CF2" s="9"/>
+      <c r="CG2" s="9"/>
+      <c r="CH2" s="9"/>
+      <c r="CI2" s="9"/>
+      <c r="CJ2" s="9"/>
+      <c r="CK2" s="9"/>
+      <c r="CL2" s="9"/>
+      <c r="CM2" s="9"/>
+      <c r="CN2" s="9"/>
+      <c r="CO2" s="9"/>
+      <c r="CP2" s="9"/>
+      <c r="CQ2" s="9"/>
+      <c r="CR2" s="9"/>
+      <c r="CS2" s="9"/>
+      <c r="CT2" s="9"/>
+      <c r="CU2" s="9"/>
+      <c r="CV2" s="9"/>
+      <c r="CW2" s="9"/>
+      <c r="CX2" s="9"/>
+      <c r="CY2" s="9"/>
+      <c r="CZ2" s="9"/>
+      <c r="DA2" s="9"/>
+      <c r="DB2" s="9"/>
+      <c r="DC2" s="9"/>
+      <c r="DD2" s="9"/>
+      <c r="DE2" s="9"/>
+      <c r="DF2" s="9"/>
+      <c r="DG2" s="9"/>
+      <c r="DH2" s="9"/>
+      <c r="DI2" s="9"/>
+      <c r="DJ2" s="9"/>
+      <c r="DK2" s="9"/>
+      <c r="DL2" s="9"/>
+      <c r="DM2" s="9"/>
+      <c r="DN2" s="9"/>
+      <c r="DO2" s="9"/>
+      <c r="DP2" s="9"/>
+      <c r="DQ2" s="9"/>
+      <c r="DR2" s="9"/>
+      <c r="DS2" s="9"/>
+      <c r="DT2" s="9"/>
+      <c r="DU2" s="9"/>
+      <c r="DV2" s="9"/>
+      <c r="DW2" s="9"/>
+      <c r="DX2" s="9"/>
+      <c r="DY2" s="9"/>
+      <c r="DZ2" s="9"/>
+      <c r="EA2" s="9"/>
+      <c r="EB2" s="9"/>
+      <c r="EC2" s="9"/>
+      <c r="ED2" s="9"/>
+      <c r="EE2" s="9"/>
+      <c r="EF2" s="9"/>
+      <c r="EG2" s="9"/>
+      <c r="EH2" s="9"/>
+      <c r="EI2" s="9"/>
+      <c r="EJ2" s="9"/>
+      <c r="EK2" s="9"/>
+      <c r="EL2" s="9"/>
+      <c r="EM2" s="9"/>
+      <c r="EN2" s="9"/>
+      <c r="EO2" s="9"/>
+      <c r="EP2" s="9"/>
+      <c r="EQ2" s="9"/>
+      <c r="ER2" s="9"/>
+      <c r="ES2" s="9"/>
+      <c r="ET2" s="9"/>
+      <c r="EU2" s="9"/>
+      <c r="EV2" s="9"/>
+      <c r="EW2" s="9"/>
+      <c r="EX2" s="9"/>
+      <c r="EY2" s="9"/>
+      <c r="EZ2" s="9"/>
+      <c r="FA2" s="9"/>
+      <c r="FB2" s="9"/>
+      <c r="FC2" s="9"/>
+      <c r="FD2" s="9"/>
+      <c r="FE2" s="9"/>
+      <c r="FF2" s="9"/>
+      <c r="FG2" s="9"/>
+      <c r="FH2" s="9"/>
+      <c r="FI2" s="9"/>
+      <c r="FJ2" s="9"/>
+      <c r="FK2" s="9"/>
+      <c r="FL2" s="9"/>
+      <c r="FM2" s="9"/>
+      <c r="FN2" s="9"/>
+      <c r="FO2" s="9"/>
+      <c r="FP2" s="9"/>
+      <c r="FQ2" s="9"/>
+      <c r="FR2" s="9"/>
+      <c r="FS2" s="9"/>
+      <c r="FT2" s="9"/>
+      <c r="FU2" s="9"/>
+      <c r="FV2" s="9"/>
+      <c r="FW2" s="9"/>
+      <c r="FX2" s="9"/>
+      <c r="FY2" s="9"/>
+      <c r="FZ2" s="9"/>
+      <c r="GA2" s="9"/>
+      <c r="GB2" s="9"/>
+      <c r="GC2" s="9"/>
+      <c r="GD2" s="9"/>
+      <c r="GE2" s="9"/>
+      <c r="GF2" s="9"/>
+      <c r="GG2" s="9"/>
+      <c r="GH2" s="9"/>
+      <c r="GI2" s="9"/>
+      <c r="GJ2" s="9"/>
+      <c r="GK2" s="9"/>
+      <c r="GL2" s="9"/>
+      <c r="GM2" s="9"/>
+      <c r="GN2" s="9"/>
+      <c r="GO2" s="9"/>
+      <c r="GP2" s="9"/>
+      <c r="GQ2" s="9"/>
+      <c r="GR2" s="9"/>
+      <c r="GS2" s="9"/>
+      <c r="GT2" s="9"/>
+      <c r="GU2" s="9"/>
+      <c r="GV2" s="9"/>
+      <c r="GW2" s="9"/>
+      <c r="GX2" s="9"/>
+      <c r="GY2" s="9"/>
+      <c r="GZ2" s="9"/>
+      <c r="HA2" s="9"/>
+      <c r="HB2" s="9"/>
+      <c r="HC2" s="9"/>
+      <c r="HD2" s="9"/>
+      <c r="HE2" s="9"/>
+      <c r="HF2" s="9"/>
+      <c r="HG2" s="9"/>
+      <c r="HH2" s="9"/>
+      <c r="HI2" s="9"/>
+      <c r="HJ2" s="9"/>
+      <c r="HK2" s="9"/>
+      <c r="HL2" s="9"/>
+      <c r="HM2" s="9"/>
+      <c r="HN2" s="9"/>
+      <c r="HO2" s="9"/>
+      <c r="HP2" s="9"/>
+      <c r="HQ2" s="9"/>
+      <c r="HR2" s="9"/>
+      <c r="HS2" s="9"/>
+      <c r="HT2" s="9"/>
+      <c r="HU2" s="9"/>
+      <c r="HV2" s="9"/>
+      <c r="HW2" s="9"/>
+      <c r="HX2" s="9"/>
+      <c r="HY2" s="9"/>
+      <c r="HZ2" s="9"/>
+      <c r="IA2" s="9"/>
+      <c r="IB2" s="9"/>
+      <c r="IC2" s="9"/>
+      <c r="ID2" s="9"/>
+      <c r="IE2" s="9"/>
+      <c r="IF2" s="9"/>
+      <c r="IG2" s="9"/>
+      <c r="IH2" s="9"/>
+      <c r="II2" s="9"/>
+      <c r="IJ2" s="9"/>
+      <c r="IK2" s="9"/>
+      <c r="IL2" s="9"/>
+      <c r="IM2" s="9"/>
+      <c r="IN2" s="9"/>
+      <c r="IO2" s="9"/>
+      <c r="IP2" s="9"/>
+      <c r="IQ2" s="9"/>
+      <c r="IR2" s="9"/>
+      <c r="IS2" s="9"/>
+      <c r="IT2" s="9"/>
+      <c r="IU2" s="9"/>
+      <c r="IV2" s="9"/>
+      <c r="IW2" s="9"/>
+      <c r="IX2" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2233,12 +2297,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="13.8" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="12" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="13.8" customHeight="1">
-      <c r="A2" s="15"/>
+      <c r="A2" s="13"/>
     </row>
     <row r="3" spans="1:1" ht="16.05" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -2284,12 +2348,12 @@
       <c r="A11" s="3"/>
     </row>
     <row r="12" spans="1:1" ht="13.8" customHeight="1">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="14" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="12" customHeight="1">
-      <c r="A13" s="17"/>
+      <c r="A13" s="15"/>
     </row>
     <row r="14" spans="1:1" ht="16.05" customHeight="1">
       <c r="A14" s="4" t="s">

</xml_diff>